<commit_message>
M5: v0.1.0 docs (README, multi-agent build story, CHANGELOG, release notes), MIS F1 numeric, cross-OS PBIP test fix
Supervisor-Approval: auto: pre-approved by user 2026-10-26 (M3-M5 relayed 10:06 PM IST)
</commit_message>
<xml_diff>
--- a/bi/data/mis.xlsx
+++ b/bi/data/mis.xlsx
@@ -26,9 +26,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##,##0"/>
     <numFmt numFmtId="165" formatCode="#,##,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -62,11 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,10 +509,8 @@
           <t>Extraction macro F1</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>